<commit_message>
Add JSON backup + restore as a full-fidelity data safety net
- 'Backup (JSON)' downloads every item (incl. image URLs) as a dated
  poda_backup_YYYY-MM-DD.json envelope.
- 'Restore' reads such a file and upserts the items back into the DB
  (accepts the envelope or a bare array; skips items without an id;
  confirms before overwriting).
Unlike the Excel export (read-only reporting), a backup is re-importable
to recover from accidental deletes or a lost project.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/poda_capital_inventory.xlsx
+++ b/poda_capital_inventory.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="152">
   <si>
     <t>PODA CAPITAL</t>
   </si>
@@ -99,6 +99,9 @@
     <t>SOLD</t>
   </si>
   <si>
+    <t>Pants</t>
+  </si>
+  <si>
     <t>NOTES / CURRENT FOCUS</t>
   </si>
   <si>
@@ -228,6 +231,42 @@
     <t>NOTES</t>
   </si>
   <si>
+    <t>PODA-26-ERICEMAN-UNK-PANTS-001</t>
+  </si>
+  <si>
+    <t>Eric Emanuel</t>
+  </si>
+  <si>
+    <t>Eric Emanuel Purple Pants</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Purple</t>
+  </si>
+  <si>
+    <t>Very Good</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-06-14</t>
+  </si>
+  <si>
+    <t>2nd Street</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>2026-06-18</t>
+  </si>
+  <si>
+    <t>www.grailed.com</t>
+  </si>
+  <si>
     <t>PODA CAPITAL — TRANSACTION LOG</t>
   </si>
   <si>
@@ -258,6 +297,12 @@
     <t>DAYS HELD</t>
   </si>
   <si>
+    <t>BUY</t>
+  </si>
+  <si>
+    <t>Eric Emanuel Eric Emanuel Purple Pants</t>
+  </si>
+  <si>
     <t>TOTALS</t>
   </si>
   <si>
@@ -421,9 +466,6 @@
   </si>
   <si>
     <t>Archive</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
   <si>
     <t>Assumed Fee % (avg)</t>
@@ -509,7 +551,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -556,6 +598,11 @@
         <fgColor rgb="FFD9E2EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -584,7 +631,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -649,11 +696,32 @@
     <xf numFmtId="164" fontId="8" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1024,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1077,15 +1145,15 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="6">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F7" s="6"/>
     </row>
@@ -1141,7 +1209,7 @@
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="5"/>
     </row>
@@ -1212,13 +1280,13 @@
         <v>21</v>
       </c>
       <c r="B18" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" s="15">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="D18" s="15">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E18" s="15">
         <v>0</v>
@@ -1252,13 +1320,13 @@
         <v>23</v>
       </c>
       <c r="B20" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" s="21">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="D20" s="21">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E20" s="21">
         <v>0</v>
@@ -1297,41 +1365,61 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="22" t="s">
+      <c r="B24" s="23">
+        <v>1</v>
+      </c>
+      <c r="C24" s="24">
+        <v>150</v>
+      </c>
+      <c r="D24" s="24">
+        <v>200</v>
+      </c>
+      <c r="E24" s="23">
+        <v>0</v>
+      </c>
+      <c r="F24" s="24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="22"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
+      <c r="A27" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="22"/>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -1360,8 +1448,8 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A26:F28"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A27:F29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1370,7 +1458,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF4"/>
+  <dimension ref="A1:AF5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1400,7 +1488,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1436,7 +1524,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1471,149 +1559,247 @@
       <c r="AF2" s="2"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23" t="s">
+      <c r="A3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23" t="s">
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="M3" s="23"/>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="23" t="s">
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="Q3" s="23"/>
-      <c r="R3" s="23"/>
-      <c r="S3" s="23" t="s">
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="T3" s="23"/>
-      <c r="U3" s="23"/>
-      <c r="V3" s="23"/>
-      <c r="W3" s="23"/>
-      <c r="X3" s="23"/>
-      <c r="Y3" s="23" t="s">
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="Z3" s="23"/>
-      <c r="AA3" s="23"/>
-      <c r="AB3" s="23"/>
-      <c r="AC3" s="23" t="s">
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="AD3" s="23"/>
-      <c r="AE3" s="23"/>
-      <c r="AF3" s="23"/>
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="26"/>
+      <c r="AC3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD3" s="26"/>
+      <c r="AE3" s="26"/>
+      <c r="AF3" s="26"/>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="V4" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="X4" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Z4" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AA4" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AB4" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AC4" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AD4" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AE4" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AF4" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L5" s="27">
+        <v>150</v>
+      </c>
+      <c r="M5" s="27">
+        <v>0</v>
+      </c>
+      <c r="N5" s="27">
+        <v>0</v>
+      </c>
+      <c r="O5" s="27">
+        <v>150</v>
+      </c>
+      <c r="P5" s="27">
+        <v>200</v>
+      </c>
+      <c r="Q5" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="R5" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="S5" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="T5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="U5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="V5" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="W5" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="X5" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="Y5" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z5" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA5" s="13">
+        <v>6</v>
+      </c>
+      <c r="AB5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="AD5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="AE5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="AF5" s="13" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1635,7 +1821,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1651,7 +1837,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1665,7 +1851,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1679,51 +1865,83 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="G3" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="29">
+        <v>150</v>
+      </c>
+      <c r="G4" s="29">
+        <v>0</v>
+      </c>
+      <c r="H4" s="29">
+        <v>-150</v>
+      </c>
+      <c r="I4" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="26">
-        <v>0</v>
-      </c>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
+      <c r="J4" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="33">
+        <v>-150</v>
+      </c>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1755,7 +1973,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1772,7 +1990,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1789,43 +2007,43 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1856,7 +2074,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1869,7 +2087,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1882,31 +2100,31 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1931,265 +2149,265 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4" s="28">
-        <v>0</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>104</v>
+      <c r="A4" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="35">
+        <v>1</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="30">
-        <v>0</v>
-      </c>
-      <c r="C5" s="29" t="s">
-        <v>106</v>
+      <c r="A5" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="37">
+        <v>150</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="B6" s="30">
-        <v>0</v>
-      </c>
-      <c r="C6" s="29" t="s">
-        <v>108</v>
+      <c r="A6" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="37">
+        <v>200</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="B7" s="30">
-        <v>0</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>110</v>
+      <c r="A7" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="37">
+        <v>0</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B8" s="30">
-        <v>0</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>112</v>
+      <c r="A8" s="34" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="37">
+        <v>0</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="B9" s="31">
-        <v>0</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>114</v>
+      <c r="A9" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" s="38">
+        <v>0</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="B10" s="32">
-        <v>0</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>116</v>
+      <c r="A10" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="39">
+        <v>0</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="31">
-        <v>0</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>118</v>
+      <c r="A11" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="38">
+        <v>0</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="B12" s="28">
-        <v>0</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>120</v>
+      <c r="A12" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" s="35">
+        <v>1</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="B13" s="28">
-        <v>0</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>122</v>
+      <c r="A13" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" s="35">
+        <v>0</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="B17" s="31">
+      <c r="A17" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="B17" s="38">
         <v>0.09</v>
       </c>
-      <c r="C17" s="29" t="s">
-        <v>127</v>
+      <c r="C17" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="B18" s="31">
+      <c r="A18" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="B18" s="38">
         <v>0.1</v>
       </c>
-      <c r="C18" s="29" t="s">
-        <v>127</v>
+      <c r="C18" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="B19" s="31">
+      <c r="A19" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" s="38">
         <v>0.13</v>
       </c>
-      <c r="C19" s="29" t="s">
-        <v>127</v>
+      <c r="C19" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="B20" s="31">
+      <c r="A20" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="B20" s="38">
         <v>0.03</v>
       </c>
-      <c r="C20" s="29" t="s">
-        <v>127</v>
+      <c r="C20" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="31">
+      <c r="A21" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="B21" s="38">
         <v>0.15</v>
       </c>
-      <c r="C21" s="29" t="s">
-        <v>127</v>
+      <c r="C21" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B22" s="31">
+      <c r="A22" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="38">
         <v>0.09</v>
       </c>
-      <c r="C22" s="29" t="s">
-        <v>127</v>
+      <c r="C22" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="B23" s="31">
+      <c r="A23" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="B23" s="38">
         <v>0.095</v>
       </c>
-      <c r="C23" s="29" t="s">
-        <v>127</v>
+      <c r="C23" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="27" t="s">
-        <v>134</v>
-      </c>
-      <c r="B24" s="31">
+      <c r="A24" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="B24" s="38">
         <v>0.1</v>
       </c>
-      <c r="C24" s="29" t="s">
-        <v>127</v>
+      <c r="C24" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="B25" s="31">
+      <c r="A25" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="38">
         <v>0.1</v>
       </c>
-      <c r="C25" s="29" t="s">
-        <v>127</v>
+      <c r="C25" s="36" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="B26" s="33">
+        <v>150</v>
+      </c>
+      <c r="B26" s="40">
         <v>0.098</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Footer social links, drop measurements, prominent platform buy button
1. Footer: make Instagram + X real links (open in new tab) across all
   four public pages; remove the dead Substack icon. Add hover state.
2. Remove measurements capture: drop the dormant measurements field
   from the item schema and the PIT TO PIT / SHOULDER / LENGTH columns
   from the Excel export (regenerated the empty template).
3. Item detail page: replace the small 'View listing' text link with a
   prominent 'Shop on {Platform}' button (Grailed/Depop/etc. detected
   from the listing URL). Closet cards use the same platform-aware label.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/poda_capital_inventory.xlsx
+++ b/poda_capital_inventory.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="134">
   <si>
     <t>PODA CAPITAL</t>
   </si>
@@ -99,9 +99,6 @@
     <t>SOLD</t>
   </si>
   <si>
-    <t>Pants</t>
-  </si>
-  <si>
     <t>NOTES / CURRENT FOCUS</t>
   </si>
   <si>
@@ -132,7 +129,7 @@
     <t>ANALYTICS</t>
   </si>
   <si>
-    <t>MEASUREMENTS</t>
+    <t>NOTES</t>
   </si>
   <si>
     <t>ITEM ID</t>
@@ -219,253 +216,202 @@
     <t>DAYS TO SELL</t>
   </si>
   <si>
-    <t>PIT TO PIT</t>
-  </si>
-  <si>
-    <t>SHOULDER</t>
-  </si>
-  <si>
-    <t>LENGTH</t>
-  </si>
-  <si>
-    <t>NOTES</t>
-  </si>
-  <si>
-    <t>PODA-26-ERICEMAN-UNK-PANTS-001</t>
-  </si>
-  <si>
-    <t>Eric Emanuel</t>
-  </si>
-  <si>
-    <t>Eric Emanuel Purple Pants</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>Purple</t>
-  </si>
-  <si>
-    <t>Very Good</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2026-06-14</t>
-  </si>
-  <si>
-    <t>2nd Street</t>
+    <t>PODA CAPITAL — TRANSACTION LOG</t>
+  </si>
+  <si>
+    <t>Every acquisition and sale, in date order.</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>ITEM</t>
+  </si>
+  <si>
+    <t>PLATFORM</t>
+  </si>
+  <si>
+    <t>GROSS AMOUNT</t>
+  </si>
+  <si>
+    <t>SHIPPING</t>
+  </si>
+  <si>
+    <t>NET AMOUNT</t>
+  </si>
+  <si>
+    <t>DAYS HELD</t>
+  </si>
+  <si>
+    <t>TOTALS</t>
+  </si>
+  <si>
+    <t>PODA CAPITAL — SOURCING PIPELINE</t>
+  </si>
+  <si>
+    <t>Items you're watching, before they enter the closet.</t>
+  </si>
+  <si>
+    <t>DATE SPOTTED</t>
+  </si>
+  <si>
+    <t>ASKING PRICE</t>
+  </si>
+  <si>
+    <t>COMP LOW</t>
+  </si>
+  <si>
+    <t>COMP MID</t>
+  </si>
+  <si>
+    <t>COMP HIGH</t>
+  </si>
+  <si>
+    <t>TARGET BUY</t>
+  </si>
+  <si>
+    <t>EST. LIST</t>
+  </si>
+  <si>
+    <t>EST. PROFIT</t>
+  </si>
+  <si>
+    <t>EST. MARGIN</t>
+  </si>
+  <si>
+    <t>PODA CAPITAL — MARKET COMPS</t>
+  </si>
+  <si>
+    <t>Sold-listing comparables backing your pricing.</t>
+  </si>
+  <si>
+    <t>COMP TYPE</t>
+  </si>
+  <si>
+    <t>SOLD PRICE</t>
+  </si>
+  <si>
+    <t>RELEVANCE</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>PODA CAPITAL — CALCULATIONS ENGINE</t>
+  </si>
+  <si>
+    <t>Definitions feeding the Overview sheet.</t>
+  </si>
+  <si>
+    <t>METRIC</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>DEFINITION</t>
+  </si>
+  <si>
+    <t>Total Items</t>
+  </si>
+  <si>
+    <t>All items with an ID</t>
+  </si>
+  <si>
+    <t>Inventory at Cost (active)</t>
+  </si>
+  <si>
+    <t>Cost basis of Closet + Listed items</t>
+  </si>
+  <si>
+    <t>Total Listed Value</t>
+  </si>
+  <si>
+    <t>Sum of list prices for Listed items</t>
+  </si>
+  <si>
+    <t>Realized Revenue</t>
+  </si>
+  <si>
+    <t>Sum of sale prices for Sold items</t>
+  </si>
+  <si>
+    <t>Realized Net Profit</t>
+  </si>
+  <si>
+    <t>Net profit after fees + shipping</t>
+  </si>
+  <si>
+    <t>Sell-Through Rate</t>
+  </si>
+  <si>
+    <t>Sold / (Sold + Listed)</t>
+  </si>
+  <si>
+    <t>Avg Days to Sell</t>
+  </si>
+  <si>
+    <t>Average of days-to-sell for Sold items</t>
+  </si>
+  <si>
+    <t>Avg Net Margin</t>
+  </si>
+  <si>
+    <t>Total net profit / total revenue</t>
+  </si>
+  <si>
+    <t>Items Listed</t>
+  </si>
+  <si>
+    <t>Items currently Listed</t>
+  </si>
+  <si>
+    <t>Items Sold</t>
+  </si>
+  <si>
+    <t>Items currently Sold</t>
+  </si>
+  <si>
+    <t>FEE ASSUMPTIONS  (update as needed)</t>
+  </si>
+  <si>
+    <t>FEE %</t>
+  </si>
+  <si>
+    <t>NOTE</t>
+  </si>
+  <si>
+    <t>Grailed</t>
+  </si>
+  <si>
+    <t>Standard all-in seller fee</t>
+  </si>
+  <si>
+    <t>Depop</t>
+  </si>
+  <si>
+    <t>eBay</t>
+  </si>
+  <si>
+    <t>Instagram</t>
+  </si>
+  <si>
+    <t>Vestiaire</t>
+  </si>
+  <si>
+    <t>StockX</t>
+  </si>
+  <si>
+    <t>GOAT</t>
+  </si>
+  <si>
+    <t>Archive</t>
   </si>
   <si>
     <t>Other</t>
-  </si>
-  <si>
-    <t>2026-06-18</t>
-  </si>
-  <si>
-    <t>www.grailed.com</t>
-  </si>
-  <si>
-    <t>PODA CAPITAL — TRANSACTION LOG</t>
-  </si>
-  <si>
-    <t>Every acquisition and sale, in date order.</t>
-  </si>
-  <si>
-    <t>DATE</t>
-  </si>
-  <si>
-    <t>TYPE</t>
-  </si>
-  <si>
-    <t>ITEM</t>
-  </si>
-  <si>
-    <t>PLATFORM</t>
-  </si>
-  <si>
-    <t>GROSS AMOUNT</t>
-  </si>
-  <si>
-    <t>SHIPPING</t>
-  </si>
-  <si>
-    <t>NET AMOUNT</t>
-  </si>
-  <si>
-    <t>DAYS HELD</t>
-  </si>
-  <si>
-    <t>BUY</t>
-  </si>
-  <si>
-    <t>Eric Emanuel Eric Emanuel Purple Pants</t>
-  </si>
-  <si>
-    <t>TOTALS</t>
-  </si>
-  <si>
-    <t>PODA CAPITAL — SOURCING PIPELINE</t>
-  </si>
-  <si>
-    <t>Items you're watching, before they enter the closet.</t>
-  </si>
-  <si>
-    <t>DATE SPOTTED</t>
-  </si>
-  <si>
-    <t>ASKING PRICE</t>
-  </si>
-  <si>
-    <t>COMP LOW</t>
-  </si>
-  <si>
-    <t>COMP MID</t>
-  </si>
-  <si>
-    <t>COMP HIGH</t>
-  </si>
-  <si>
-    <t>TARGET BUY</t>
-  </si>
-  <si>
-    <t>EST. LIST</t>
-  </si>
-  <si>
-    <t>EST. PROFIT</t>
-  </si>
-  <si>
-    <t>EST. MARGIN</t>
-  </si>
-  <si>
-    <t>PODA CAPITAL — MARKET COMPS</t>
-  </si>
-  <si>
-    <t>Sold-listing comparables backing your pricing.</t>
-  </si>
-  <si>
-    <t>COMP TYPE</t>
-  </si>
-  <si>
-    <t>SOLD PRICE</t>
-  </si>
-  <si>
-    <t>RELEVANCE</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>PODA CAPITAL — CALCULATIONS ENGINE</t>
-  </si>
-  <si>
-    <t>Definitions feeding the Overview sheet.</t>
-  </si>
-  <si>
-    <t>METRIC</t>
-  </si>
-  <si>
-    <t>VALUE</t>
-  </si>
-  <si>
-    <t>DEFINITION</t>
-  </si>
-  <si>
-    <t>Total Items</t>
-  </si>
-  <si>
-    <t>All items with an ID</t>
-  </si>
-  <si>
-    <t>Inventory at Cost (active)</t>
-  </si>
-  <si>
-    <t>Cost basis of Closet + Listed items</t>
-  </si>
-  <si>
-    <t>Total Listed Value</t>
-  </si>
-  <si>
-    <t>Sum of list prices for Listed items</t>
-  </si>
-  <si>
-    <t>Realized Revenue</t>
-  </si>
-  <si>
-    <t>Sum of sale prices for Sold items</t>
-  </si>
-  <si>
-    <t>Realized Net Profit</t>
-  </si>
-  <si>
-    <t>Net profit after fees + shipping</t>
-  </si>
-  <si>
-    <t>Sell-Through Rate</t>
-  </si>
-  <si>
-    <t>Sold / (Sold + Listed)</t>
-  </si>
-  <si>
-    <t>Avg Days to Sell</t>
-  </si>
-  <si>
-    <t>Average of days-to-sell for Sold items</t>
-  </si>
-  <si>
-    <t>Avg Net Margin</t>
-  </si>
-  <si>
-    <t>Total net profit / total revenue</t>
-  </si>
-  <si>
-    <t>Items Listed</t>
-  </si>
-  <si>
-    <t>Items currently Listed</t>
-  </si>
-  <si>
-    <t>Items Sold</t>
-  </si>
-  <si>
-    <t>Items currently Sold</t>
-  </si>
-  <si>
-    <t>FEE ASSUMPTIONS  (update as needed)</t>
-  </si>
-  <si>
-    <t>FEE %</t>
-  </si>
-  <si>
-    <t>NOTE</t>
-  </si>
-  <si>
-    <t>Grailed</t>
-  </si>
-  <si>
-    <t>Standard all-in seller fee</t>
-  </si>
-  <si>
-    <t>Depop</t>
-  </si>
-  <si>
-    <t>eBay</t>
-  </si>
-  <si>
-    <t>Instagram</t>
-  </si>
-  <si>
-    <t>Vestiaire</t>
-  </si>
-  <si>
-    <t>StockX</t>
-  </si>
-  <si>
-    <t>GOAT</t>
-  </si>
-  <si>
-    <t>Archive</t>
   </si>
   <si>
     <t>Assumed Fee % (avg)</t>
@@ -551,7 +497,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -598,11 +544,6 @@
         <fgColor rgb="FFD9E2EC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -631,7 +572,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -696,32 +637,11 @@
     <xf numFmtId="164" fontId="8" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1092,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1145,15 +1065,15 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="6">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F7" s="6"/>
     </row>
@@ -1209,7 +1129,7 @@
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="5"/>
     </row>
@@ -1280,13 +1200,13 @@
         <v>21</v>
       </c>
       <c r="B18" s="14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="15">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="D18" s="15">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="E18" s="15">
         <v>0</v>
@@ -1320,13 +1240,13 @@
         <v>23</v>
       </c>
       <c r="B20" s="20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" s="21">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="D20" s="21">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="E20" s="21">
         <v>0</v>
@@ -1365,61 +1285,41 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="22" t="s">
+    <row r="25" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="23">
-        <v>1</v>
-      </c>
-      <c r="C24" s="24">
-        <v>150</v>
-      </c>
-      <c r="D24" s="24">
-        <v>200</v>
-      </c>
-      <c r="E24" s="23">
-        <v>0</v>
-      </c>
-      <c r="F24" s="24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="25"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -1448,8 +1348,8 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A27:F29"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A26:F28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1458,7 +1358,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF5"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1483,12 +1383,12 @@
     <col min="22" max="23" width="11" customWidth="1"/>
     <col min="24" max="25" width="12" customWidth="1"/>
     <col min="26" max="28" width="11" customWidth="1"/>
-    <col min="32" max="32" width="30" customWidth="1"/>
+    <col min="29" max="29" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1518,13 +1418,10 @@
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
-      <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-      <c r="AF1" s="1"/>
-    </row>
-    <row r="2" ht="16" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1554,265 +1451,151 @@
       <c r="AA2" s="2"/>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
-      <c r="AD2" s="2"/>
-      <c r="AE2" s="2"/>
-      <c r="AF2" s="2"/>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26" t="s">
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26" t="s">
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26" t="s">
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26" t="s">
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
+      <c r="Y3" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="T3" s="26"/>
-      <c r="U3" s="26"/>
-      <c r="V3" s="26"/>
-      <c r="W3" s="26"/>
-      <c r="X3" s="26"/>
-      <c r="Y3" s="26" t="s">
+      <c r="Z3" s="23"/>
+      <c r="AA3" s="23"/>
+      <c r="AB3" s="23"/>
+      <c r="AC3" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="Z3" s="26"/>
-      <c r="AA3" s="26"/>
-      <c r="AB3" s="26"/>
-      <c r="AC3" s="26" t="s">
+    </row>
+    <row r="4" ht="26" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="AD3" s="26"/>
-      <c r="AE3" s="26"/>
-      <c r="AF3" s="26"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="B4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="L4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="O4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="P4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="Q4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="Q4" s="9" t="s">
+      <c r="R4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="R4" s="9" t="s">
+      <c r="S4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="T4" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="T4" s="9" t="s">
+      <c r="U4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="U4" s="9" t="s">
+      <c r="V4" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="V4" s="9" t="s">
+      <c r="W4" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="W4" s="9" t="s">
+      <c r="X4" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="X4" s="9" t="s">
+      <c r="Y4" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="Y4" s="9" t="s">
+      <c r="Z4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="Z4" s="9" t="s">
+      <c r="AA4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="AA4" s="9" t="s">
+      <c r="AB4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="AB4" s="9" t="s">
-        <v>66</v>
-      </c>
       <c r="AC4" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD4" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="AE4" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="AF4" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="L5" s="27">
-        <v>150</v>
-      </c>
-      <c r="M5" s="27">
-        <v>0</v>
-      </c>
-      <c r="N5" s="27">
-        <v>0</v>
-      </c>
-      <c r="O5" s="27">
-        <v>150</v>
-      </c>
-      <c r="P5" s="27">
-        <v>200</v>
-      </c>
-      <c r="Q5" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="R5" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="S5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="T5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="U5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="V5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="W5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="X5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="Y5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="Z5" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA5" s="13">
-        <v>6</v>
-      </c>
-      <c r="AB5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AC5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AD5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AE5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AF5" s="13" t="s">
-        <v>77</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="A2:AF2"/>
+  <mergeCells count="8">
+    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A2:AC2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="L3:O3"/>
     <mergeCell ref="P3:R3"/>
     <mergeCell ref="S3:X3"/>
     <mergeCell ref="Y3:AB3"/>
-    <mergeCell ref="AC3:AF3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1821,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1837,7 +1620,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1851,7 +1634,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1865,83 +1648,51 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="F4" s="29">
-        <v>150</v>
-      </c>
-      <c r="G4" s="29">
-        <v>0</v>
-      </c>
-      <c r="H4" s="29">
-        <v>-150</v>
-      </c>
-      <c r="I4" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
-        <v>95</v>
-      </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="33">
-        <v>-150</v>
-      </c>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="A4" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="26">
+        <v>0</v>
+      </c>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1973,7 +1724,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1990,7 +1741,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2007,43 +1758,43 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2074,7 +1825,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2087,7 +1838,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2100,31 +1851,31 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2149,265 +1900,265 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="28">
+        <v>0</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="30">
+        <v>0</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="30">
+        <v>0</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="30">
+        <v>0</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="30">
+        <v>0</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="31">
+        <v>0</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" s="32">
+        <v>0</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="31">
+        <v>0</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B12" s="28">
+        <v>0</v>
+      </c>
+      <c r="C12" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="9" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="27" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="34" t="s">
+      <c r="B13" s="28">
+        <v>0</v>
+      </c>
+      <c r="C13" s="29" t="s">
         <v>118</v>
-      </c>
-      <c r="B4" s="35">
-        <v>1</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="34" t="s">
-        <v>120</v>
-      </c>
-      <c r="B5" s="37">
-        <v>150</v>
-      </c>
-      <c r="C5" s="36" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" s="37">
-        <v>200</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="B7" s="37">
-        <v>0</v>
-      </c>
-      <c r="C7" s="36" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" s="37">
-        <v>0</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="B9" s="38">
-        <v>0</v>
-      </c>
-      <c r="C9" s="36" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B10" s="39">
-        <v>0</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B11" s="38">
-        <v>0</v>
-      </c>
-      <c r="C11" s="36" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="B12" s="35">
-        <v>1</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="B13" s="35">
-        <v>0</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="B17" s="38">
+      <c r="A17" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" s="31">
         <v>0.09</v>
       </c>
-      <c r="C17" s="36" t="s">
-        <v>142</v>
+      <c r="C17" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="B18" s="38">
+      <c r="A18" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="31">
         <v>0.1</v>
       </c>
-      <c r="C18" s="36" t="s">
-        <v>142</v>
+      <c r="C18" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="B19" s="38">
+      <c r="A19" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="B19" s="31">
         <v>0.13</v>
       </c>
-      <c r="C19" s="36" t="s">
-        <v>142</v>
+      <c r="C19" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="B20" s="38">
+      <c r="A20" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="B20" s="31">
         <v>0.03</v>
       </c>
-      <c r="C20" s="36" t="s">
-        <v>142</v>
+      <c r="C20" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="34" t="s">
-        <v>146</v>
-      </c>
-      <c r="B21" s="38">
+      <c r="A21" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21" s="31">
         <v>0.15</v>
       </c>
-      <c r="C21" s="36" t="s">
-        <v>142</v>
+      <c r="C21" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="34" t="s">
-        <v>147</v>
-      </c>
-      <c r="B22" s="38">
+      <c r="A22" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B22" s="31">
         <v>0.09</v>
       </c>
-      <c r="C22" s="36" t="s">
-        <v>142</v>
+      <c r="C22" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="B23" s="38">
+      <c r="A23" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="31">
         <v>0.095</v>
       </c>
-      <c r="C23" s="36" t="s">
-        <v>142</v>
+      <c r="C23" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="34" t="s">
-        <v>149</v>
-      </c>
-      <c r="B24" s="38">
+      <c r="A24" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="31">
         <v>0.1</v>
       </c>
-      <c r="C24" s="36" t="s">
-        <v>142</v>
+      <c r="C24" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="34" t="s">
-        <v>80</v>
-      </c>
-      <c r="B25" s="38">
+      <c r="A25" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="31">
         <v>0.1</v>
       </c>
-      <c r="C25" s="36" t="s">
-        <v>142</v>
+      <c r="C25" s="29" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="B26" s="40">
+        <v>132</v>
+      </c>
+      <c r="B26" s="33">
         <v>0.098</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>